<commit_message>
Page Objects development and Excel file configuration using mapper
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\Symex\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88F49B8-DC79-4DDF-B754-318EF886DCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF38F2AB-22EF-48E0-8D21-C4D10C7285A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
   <si>
     <t>titleValidationTest</t>
   </si>
@@ -61,13 +61,115 @@
   </si>
   <si>
     <t>Symx@4322</t>
+  </si>
+  <si>
+    <t>customerCategory</t>
+  </si>
+  <si>
+    <t>riskCategory</t>
+  </si>
+  <si>
+    <t>residentType</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>materialStatus</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>middleName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>firstUnicodeName</t>
+  </si>
+  <si>
+    <t>middleUnicodeName</t>
+  </si>
+  <si>
+    <t>lastUnicodeName</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>nationality</t>
+  </si>
+  <si>
+    <t>dualNationality</t>
+  </si>
+  <si>
+    <t>countryOfBirth</t>
+  </si>
+  <si>
+    <t>placeOfBirth</t>
+  </si>
+  <si>
+    <t>phoneCode</t>
+  </si>
+  <si>
+    <t>mobileNumber</t>
+  </si>
+  <si>
+    <t>phoneNumber</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>NonResident</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Gopinath</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>gopinath@cinque.ae</t>
+  </si>
+  <si>
+    <t>Symx@14#</t>
+  </si>
+  <si>
+    <t>registerCustomer</t>
+  </si>
+  <si>
+    <t>Natural Person</t>
+  </si>
+  <si>
+    <t>UnMarried</t>
+  </si>
+  <si>
+    <t>hungary</t>
+  </si>
+  <si>
+    <t>bhutan</t>
+  </si>
+  <si>
+    <t>30/10/1999</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,6 +190,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -110,10 +218,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,16 +505,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -416,36 +547,96 @@
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -458,6 +649,65 @@
       <c r="D4" t="s">
         <v>6</v>
       </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T5" t="s">
+        <v>44</v>
+      </c>
+      <c r="U5">
+        <v>91</v>
+      </c>
+      <c r="V5">
+        <v>7550157717</v>
+      </c>
+      <c r="X5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="I7" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Page Objects development for other customer registration components
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF38F2AB-22EF-48E0-8D21-C4D10C7285A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4644AFCF-58C2-42A6-A19C-CE9EB05754BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -218,13 +218,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,7 +688,7 @@
       <c r="P5" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="Q5" s="4" t="s">
         <v>43</v>
       </c>
       <c r="S5" t="s">

</xml_diff>

<commit_message>
Methods and page objects update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks1\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4644AFCF-58C2-42A6-A19C-CE9EB05754BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B84D31-FFA8-48F8-99A8-6E97E04DE4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5340" yWindow="975" windowWidth="15360" windowHeight="6735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="70">
   <si>
     <t>titleValidationTest</t>
   </si>
@@ -163,6 +163,78 @@
   </si>
   <si>
     <t>30/10/1999</t>
+  </si>
+  <si>
+    <t>addressInUAE</t>
+  </si>
+  <si>
+    <t>poBox</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>nearestAirport</t>
+  </si>
+  <si>
+    <t>emirate</t>
+  </si>
+  <si>
+    <t>district</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>homeAddressInCountry</t>
+  </si>
+  <si>
+    <t>UAE Address</t>
+  </si>
+  <si>
+    <t>Dubai</t>
+  </si>
+  <si>
+    <t>Sharjah</t>
+  </si>
+  <si>
+    <t>Ajman</t>
+  </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Home address data</t>
+  </si>
+  <si>
+    <t>temporaryAddress</t>
+  </si>
+  <si>
+    <t>Temp address data</t>
+  </si>
+  <si>
+    <t>employer</t>
+  </si>
+  <si>
+    <t>occupation</t>
+  </si>
+  <si>
+    <t>Cinque Tecnologies</t>
+  </si>
+  <si>
+    <t>Banking Business Manager</t>
+  </si>
+  <si>
+    <t>companyType</t>
+  </si>
+  <si>
+    <t>countryOfIncorporation</t>
+  </si>
+  <si>
+    <t>dateOfEstablishment</t>
+  </si>
+  <si>
+    <t>placeOfIncorporation</t>
   </si>
 </sst>
 </file>
@@ -506,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -533,9 +605,18 @@
     <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.7109375" customWidth="1"/>
+    <col min="26" max="26" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="22.28515625" customWidth="1"/>
+    <col min="29" max="29" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -608,8 +689,53 @@
       <c r="X1" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="Y1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>63</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -623,7 +749,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -637,7 +763,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -651,7 +777,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -706,8 +832,38 @@
       <c r="X5" t="s">
         <v>38</v>
       </c>
+      <c r="AC5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD5">
+        <v>123456</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>61</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>64</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>65</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.25">
       <c r="I7" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Page objects, DTO and Mappers update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E57F97-2BD6-442B-8C24-9F36AE81FED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B74B7A1-F1DE-4467-AB5A-61F30E81DA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6855" yWindow="255" windowWidth="15360" windowHeight="6735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="98">
   <si>
     <t>titleValidationTest</t>
   </si>
@@ -316,6 +316,9 @@
   </si>
   <si>
     <t>Employee</t>
+  </si>
+  <si>
+    <t>employee</t>
   </si>
 </sst>
 </file>
@@ -663,7 +666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BD7"/>
+  <dimension ref="A1:BE7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -714,9 +717,11 @@
     <col min="53" max="53" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="11" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -885,8 +890,11 @@
       <c r="BD1" s="1" t="s">
         <v>91</v>
       </c>
+      <c r="BE1" s="1" t="s">
+        <v>97</v>
+      </c>
     </row>
-    <row r="2" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -900,7 +908,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -914,7 +922,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -928,7 +936,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1064,8 +1072,11 @@
       <c r="BD5" t="s">
         <v>96</v>
       </c>
+      <c r="BE5" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="7" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.25">
       <c r="I7" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Page objects update and reusable methods update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9AFA52-EAB1-49B1-AB80-FE52E84CCB61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5653938E-B472-4F78-BB48-53565AD5BCDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -144,9 +144,6 @@
     <t>gopinath@cinque.ae</t>
   </si>
   <si>
-    <t>registerCustomer</t>
-  </si>
-  <si>
     <t>Natural Person</t>
   </si>
   <si>
@@ -403,6 +400,9 @@
   </si>
   <si>
     <t>testdata/idimages/idimage1.jpg,testdata/idimages/idimage2.jpg</t>
+  </si>
+  <si>
+    <t>registerIndividualCustomer</t>
   </si>
 </sst>
 </file>
@@ -896,163 +896,163 @@
         <v>31</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AN1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AC1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="AW1" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="AX1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="AY1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="BD1" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="BE1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="BF1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="BP1" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="BQ1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="BR1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
@@ -1099,13 +1099,13 @@
     </row>
     <row r="5" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="B5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" t="s">
         <v>82</v>
-      </c>
-      <c r="C5" t="s">
-        <v>83</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -1114,7 +1114,7 @@
         <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
         <v>33</v>
@@ -1123,7 +1123,7 @@
         <v>34</v>
       </c>
       <c r="I5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J5" t="s">
         <v>35</v>
@@ -1132,16 +1132,16 @@
         <v>36</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S5" t="s">
         <v>37</v>
       </c>
       <c r="T5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U5">
         <v>91</v>
@@ -1153,40 +1153,40 @@
         <v>38</v>
       </c>
       <c r="AC5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AD5">
         <v>123456</v>
       </c>
       <c r="AE5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF5" t="s">
         <v>54</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AG5" t="s">
         <v>55</v>
       </c>
-      <c r="AG5" t="s">
+      <c r="AI5" t="s">
         <v>56</v>
       </c>
-      <c r="AI5" t="s">
+      <c r="AJ5" t="s">
         <v>57</v>
       </c>
-      <c r="AJ5" t="s">
-        <v>58</v>
-      </c>
       <c r="AK5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AL5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AM5" t="s">
         <v>63</v>
       </c>
-      <c r="AM5" t="s">
-        <v>64</v>
-      </c>
       <c r="AN5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AO5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AP5">
         <v>86501326</v>
@@ -1204,25 +1204,25 @@
         <v>532</v>
       </c>
       <c r="AU5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AV5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AW5">
         <v>5465415</v>
       </c>
       <c r="AX5" t="s">
+        <v>91</v>
+      </c>
+      <c r="AY5" t="s">
         <v>92</v>
       </c>
-      <c r="AY5" t="s">
+      <c r="AZ5" t="s">
         <v>93</v>
       </c>
-      <c r="AZ5" t="s">
+      <c r="BA5" t="s">
         <v>94</v>
-      </c>
-      <c r="BA5" t="s">
-        <v>95</v>
       </c>
       <c r="BB5">
         <v>6260262069</v>
@@ -1231,43 +1231,43 @@
         <v>950959651959591</v>
       </c>
       <c r="BD5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BE5" t="s">
         <v>35</v>
       </c>
       <c r="BO5" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="BP5" t="s">
         <v>35</v>
       </c>
       <c r="BQ5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="BR5">
         <v>23210652</v>
       </c>
       <c r="BS5" t="s">
+        <v>119</v>
+      </c>
+      <c r="BT5" t="s">
         <v>120</v>
       </c>
-      <c r="BT5" t="s">
+      <c r="BU5" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="BU5" s="3" t="s">
+      <c r="BV5" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="BV5" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="BW5">
         <v>26502626262</v>
       </c>
       <c r="BX5" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="BY5" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="BY5" s="3" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:77" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Customer Registration screen automation scripts completion with testing
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5653938E-B472-4F78-BB48-53565AD5BCDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06DCEA63-D5B2-447D-8B1E-66F1C7763AAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="representatives" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="219">
   <si>
     <t>titleValidationTest</t>
   </si>
@@ -135,15 +136,9 @@
     <t>Gopinath</t>
   </si>
   <si>
-    <t>K</t>
-  </si>
-  <si>
     <t>India</t>
   </si>
   <si>
-    <t>gopinath@cinque.ae</t>
-  </si>
-  <si>
     <t>Natural Person</t>
   </si>
   <si>
@@ -156,9 +151,6 @@
     <t>bhutan</t>
   </si>
   <si>
-    <t>30/10/1999</t>
-  </si>
-  <si>
     <t>addressInUAE</t>
   </si>
   <si>
@@ -270,9 +262,6 @@
     <t>Pakistan</t>
   </si>
   <si>
-    <t>gopinath</t>
-  </si>
-  <si>
     <t>Symx@14#</t>
   </si>
   <si>
@@ -403,6 +392,297 @@
   </si>
   <si>
     <t>registerIndividualCustomer</t>
+  </si>
+  <si>
+    <t>testCaseName</t>
+  </si>
+  <si>
+    <t>repOrder</t>
+  </si>
+  <si>
+    <t>representativeType</t>
+  </si>
+  <si>
+    <t>placeOfIssue</t>
+  </si>
+  <si>
+    <t>idIssueDate</t>
+  </si>
+  <si>
+    <t>idIssueCountry</t>
+  </si>
+  <si>
+    <t>relation</t>
+  </si>
+  <si>
+    <t>repIdImagePath</t>
+  </si>
+  <si>
+    <t>registerCorporateCustomer</t>
+  </si>
+  <si>
+    <t>Representative</t>
+  </si>
+  <si>
+    <t>Beneficialowner</t>
+  </si>
+  <si>
+    <t>Owner/Partner</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>Sara</t>
+  </si>
+  <si>
+    <t>Mary</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Hassan</t>
+  </si>
+  <si>
+    <t>Khan</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>23/11/1998</t>
+  </si>
+  <si>
+    <t>10/02/1997</t>
+  </si>
+  <si>
+    <t>30/03/1985</t>
+  </si>
+  <si>
+    <t>01/01/2001</t>
+  </si>
+  <si>
+    <t>Greece</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t>21/10/2022</t>
+  </si>
+  <si>
+    <t>09/07/2023</t>
+  </si>
+  <si>
+    <t>02/07/2025</t>
+  </si>
+  <si>
+    <t>01/01/2026</t>
+  </si>
+  <si>
+    <t>13/09/2029</t>
+  </si>
+  <si>
+    <t>27/04/2028</t>
+  </si>
+  <si>
+    <t>06/03/2027</t>
+  </si>
+  <si>
+    <t>08/11/2029</t>
+  </si>
+  <si>
+    <t>Benin</t>
+  </si>
+  <si>
+    <t>Chad</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>Iran</t>
+  </si>
+  <si>
+    <t>02/05/2028</t>
+  </si>
+  <si>
+    <t>04/10/2028</t>
+  </si>
+  <si>
+    <t>30/10/2030</t>
+  </si>
+  <si>
+    <t>06/08/2027</t>
+  </si>
+  <si>
+    <t>Son</t>
+  </si>
+  <si>
+    <t>Daughter</t>
+  </si>
+  <si>
+    <t>Brother</t>
+  </si>
+  <si>
+    <t>Aunt</t>
+  </si>
+  <si>
+    <t>registeredBy</t>
+  </si>
+  <si>
+    <t>Remote</t>
+  </si>
+  <si>
+    <t>Outside Freezone</t>
+  </si>
+  <si>
+    <t>Legal Entities</t>
+  </si>
+  <si>
+    <t>Resident</t>
+  </si>
+  <si>
+    <t>AlignMinds </t>
+  </si>
+  <si>
+    <t>Technologies</t>
+  </si>
+  <si>
+    <t>United Arab Emirates</t>
+  </si>
+  <si>
+    <t>Barbados</t>
+  </si>
+  <si>
+    <t>Sharjae</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Al Ain</t>
+  </si>
+  <si>
+    <t>Abudhabi</t>
+  </si>
+  <si>
+    <t>IT Services</t>
+  </si>
+  <si>
+    <t>Auction</t>
+  </si>
+  <si>
+    <t>Banking</t>
+  </si>
+  <si>
+    <t>Private Sector</t>
+  </si>
+  <si>
+    <t>Tset</t>
+  </si>
+  <si>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>Shinitha</t>
+  </si>
+  <si>
+    <t>Thomas</t>
+  </si>
+  <si>
+    <t>10/05/1989</t>
+  </si>
+  <si>
+    <t>shinithat@cinque.ae</t>
+  </si>
+  <si>
+    <t>adminalignminds@gmail.com</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>virtual assets</t>
+  </si>
+  <si>
+    <t>Corporate regn</t>
+  </si>
+  <si>
+    <t>Kochi</t>
+  </si>
+  <si>
+    <t>Trade license</t>
+  </si>
+  <si>
+    <t>representativeFirstName</t>
+  </si>
+  <si>
+    <t>representativeMiddleName</t>
+  </si>
+  <si>
+    <t>representativeLastName</t>
+  </si>
+  <si>
+    <t>representativeGender</t>
+  </si>
+  <si>
+    <t>representativeDOB</t>
+  </si>
+  <si>
+    <t>representativeNationality</t>
+  </si>
+  <si>
+    <t>representativeDualNationality</t>
+  </si>
+  <si>
+    <t>representativePhoneCode</t>
+  </si>
+  <si>
+    <t>representativePhoneNumber</t>
+  </si>
+  <si>
+    <t>representativeIdType</t>
+  </si>
+  <si>
+    <t>representativeIdNumber</t>
+  </si>
+  <si>
+    <t>visaIdExpiryDate</t>
+  </si>
+  <si>
+    <t>Aruba</t>
+  </si>
+  <si>
+    <t>place</t>
+  </si>
+  <si>
+    <t>Authorized</t>
+  </si>
+  <si>
+    <t>share</t>
+  </si>
+  <si>
+    <t>90</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>05/08/2015</t>
   </si>
 </sst>
 </file>
@@ -412,7 +692,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -440,6 +720,11 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2A2A2A"/>
+      <name val="Poppins"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -461,7 +746,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -470,6 +755,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -750,10 +1038,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BY7"/>
+  <dimension ref="A1:BZ7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -762,26 +1050,27 @@
     <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="19.7109375" customWidth="1"/>
     <col min="26" max="26" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="19.7109375" customWidth="1"/>
     <col min="29" max="29" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="20" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="18.5703125" bestFit="1" customWidth="1"/>
@@ -796,33 +1085,36 @@
     <col min="47" max="47" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="11" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="18" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="23" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="10" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="12" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="60.140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="16.140625" customWidth="1"/>
+    <col min="57" max="57" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="18" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="23" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="10" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="20" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="12" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="60.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -896,166 +1188,169 @@
         <v>31</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AN1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AC1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AU1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="AX1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="BB1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="BE1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="BM1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="BV1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="BV1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="BW1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="BX1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>117</v>
-      </c>
     </row>
-    <row r="2" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1069,7 +1364,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1083,7 +1378,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1097,15 +1392,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -1114,7 +1409,7 @@
         <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G5" t="s">
         <v>33</v>
@@ -1123,70 +1418,70 @@
         <v>34</v>
       </c>
       <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" t="s">
+        <v>190</v>
+      </c>
+      <c r="L5" t="s">
+        <v>191</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" t="s">
+        <v>36</v>
+      </c>
+      <c r="T5" t="s">
         <v>40</v>
-      </c>
-      <c r="J5" t="s">
-        <v>35</v>
-      </c>
-      <c r="L5" t="s">
-        <v>36</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="S5" t="s">
-        <v>37</v>
-      </c>
-      <c r="T5" t="s">
-        <v>42</v>
       </c>
       <c r="U5">
         <v>91</v>
       </c>
       <c r="V5">
-        <v>7550157717</v>
+        <v>8521036250</v>
       </c>
       <c r="X5" t="s">
-        <v>38</v>
+        <v>193</v>
       </c>
       <c r="AC5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="AD5">
         <v>123456</v>
       </c>
       <c r="AE5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI5" t="s">
         <v>53</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AJ5" t="s">
         <v>54</v>
       </c>
-      <c r="AG5" t="s">
-        <v>55</v>
-      </c>
-      <c r="AI5" t="s">
+      <c r="AK5" t="s">
         <v>56</v>
       </c>
-      <c r="AJ5" t="s">
-        <v>57</v>
-      </c>
-      <c r="AK5" t="s">
+      <c r="AL5" t="s">
         <v>59</v>
       </c>
-      <c r="AL5" t="s">
-        <v>62</v>
-      </c>
       <c r="AM5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="AN5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AO5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AP5">
         <v>86501326</v>
@@ -1198,31 +1493,28 @@
         <v>999</v>
       </c>
       <c r="AS5">
-        <v>6265642</v>
+        <v>5965965</v>
       </c>
       <c r="AT5">
-        <v>532</v>
+        <v>123</v>
       </c>
       <c r="AU5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AV5" t="s">
-        <v>79</v>
-      </c>
-      <c r="AW5">
-        <v>5465415</v>
+        <v>76</v>
       </c>
       <c r="AX5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="AY5" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="AZ5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="BA5" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="BB5">
         <v>6260262069</v>
@@ -1230,47 +1522,202 @@
       <c r="BC5" s="5">
         <v>950959651959591</v>
       </c>
-      <c r="BD5" t="s">
-        <v>95</v>
+      <c r="BD5" s="5" t="s">
+        <v>172</v>
       </c>
       <c r="BE5" t="s">
+        <v>91</v>
+      </c>
+      <c r="BF5" t="s">
         <v>35</v>
       </c>
-      <c r="BO5" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="BP5" t="s">
+      <c r="BP5" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="BQ5" t="s">
         <v>35</v>
       </c>
-      <c r="BQ5" t="s">
+      <c r="BR5" t="s">
+        <v>114</v>
+      </c>
+      <c r="BS5">
+        <v>75120365</v>
+      </c>
+      <c r="BT5" t="s">
+        <v>115</v>
+      </c>
+      <c r="BU5" t="s">
+        <v>116</v>
+      </c>
+      <c r="BV5" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="BW5" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="BR5">
-        <v>23210652</v>
-      </c>
-      <c r="BS5" t="s">
+      <c r="BX5">
+        <v>4102213652</v>
+      </c>
+      <c r="BY5" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="BT5" t="s">
+      <c r="BZ5" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="BU5" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="BV5" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="BW5">
-        <v>26502626262</v>
-      </c>
-      <c r="BX5" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="BY5" s="3" t="s">
-        <v>124</v>
-      </c>
     </row>
-    <row r="7" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:78" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>174</v>
+      </c>
+      <c r="G6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="L6" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>178</v>
+      </c>
+      <c r="U6">
+        <v>1</v>
+      </c>
+      <c r="V6">
+        <v>853210263</v>
+      </c>
+      <c r="X6" t="s">
+        <v>194</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>173</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>179</v>
+      </c>
+      <c r="AA6" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>180</v>
+      </c>
+      <c r="AD6">
+        <v>5145656</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>181</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>182</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>183</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>178</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>195</v>
+      </c>
+      <c r="AQ6">
+        <v>63251</v>
+      </c>
+      <c r="AR6">
+        <v>56</v>
+      </c>
+      <c r="AS6">
+        <v>956321</v>
+      </c>
+      <c r="AT6">
+        <v>36</v>
+      </c>
+      <c r="AV6" t="s">
+        <v>184</v>
+      </c>
+      <c r="AW6">
+        <v>95959652</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>197</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>198</v>
+      </c>
+      <c r="AZ6" t="s">
+        <v>89</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>90</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>189</v>
+      </c>
+      <c r="BE6" t="s">
+        <v>91</v>
+      </c>
+      <c r="BF6" t="s">
+        <v>35</v>
+      </c>
+      <c r="BG6" t="s">
+        <v>196</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>188</v>
+      </c>
+      <c r="BI6" s="5">
+        <v>596596596529656</v>
+      </c>
+      <c r="BK6" t="s">
+        <v>185</v>
+      </c>
+      <c r="BL6" t="s">
+        <v>186</v>
+      </c>
+      <c r="BM6" t="s">
+        <v>187</v>
+      </c>
+      <c r="BR6" t="s">
+        <v>199</v>
+      </c>
+      <c r="BS6">
+        <v>959165656</v>
+      </c>
+      <c r="BT6" t="s">
+        <v>178</v>
+      </c>
+      <c r="BU6" t="s">
+        <v>50</v>
+      </c>
+      <c r="BV6" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="BW6" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="BZ6" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:78" x14ac:dyDescent="0.25">
       <c r="I7" s="2"/>
     </row>
   </sheetData>
@@ -1278,4 +1725,390 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56F7CC70-8EAF-4EBB-B9F1-D1C094FBB63D}">
+  <dimension ref="A1:AR5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.140625" customWidth="1"/>
+    <col min="23" max="23" width="60.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+    </row>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="I2" t="s">
+        <v>212</v>
+      </c>
+      <c r="K2">
+        <v>243</v>
+      </c>
+      <c r="L2" s="5">
+        <v>8410236950</v>
+      </c>
+      <c r="M2" t="s">
+        <v>114</v>
+      </c>
+      <c r="N2" s="5">
+        <v>62652965</v>
+      </c>
+      <c r="O2" t="s">
+        <v>213</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="R2" t="s">
+        <v>159</v>
+      </c>
+      <c r="S2" s="5">
+        <v>32616052</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="V2" s="3"/>
+      <c r="W2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>214</v>
+      </c>
+      <c r="D3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F3" t="s">
+        <v>140</v>
+      </c>
+      <c r="G3" t="s">
+        <v>143</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I3" t="s">
+        <v>148</v>
+      </c>
+      <c r="K3">
+        <v>39</v>
+      </c>
+      <c r="L3" s="5">
+        <v>9410236950</v>
+      </c>
+      <c r="M3" t="s">
+        <v>114</v>
+      </c>
+      <c r="N3" s="5">
+        <v>8748019519</v>
+      </c>
+      <c r="O3" t="s">
+        <v>213</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="R3" t="s">
+        <v>160</v>
+      </c>
+      <c r="S3" s="5">
+        <v>740000562</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="V3" s="3"/>
+      <c r="W3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F4" t="s">
+        <v>141</v>
+      </c>
+      <c r="G4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="I4" t="s">
+        <v>149</v>
+      </c>
+      <c r="K4">
+        <v>40</v>
+      </c>
+      <c r="L4" s="5">
+        <v>1024710236</v>
+      </c>
+      <c r="M4" t="s">
+        <v>114</v>
+      </c>
+      <c r="N4" s="5">
+        <v>9595016</v>
+      </c>
+      <c r="O4" t="s">
+        <v>213</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="R4" t="s">
+        <v>161</v>
+      </c>
+      <c r="S4" s="5">
+        <v>521032154</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="V4" t="s">
+        <v>216</v>
+      </c>
+      <c r="W4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G5" t="s">
+        <v>143</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I5" t="s">
+        <v>150</v>
+      </c>
+      <c r="K5">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5">
+        <v>6012354012</v>
+      </c>
+      <c r="M5" t="s">
+        <v>114</v>
+      </c>
+      <c r="N5" s="5">
+        <v>654515332</v>
+      </c>
+      <c r="O5" t="s">
+        <v>213</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="R5" t="s">
+        <v>162</v>
+      </c>
+      <c r="S5" s="5">
+        <v>5490196</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="V5" t="s">
+        <v>217</v>
+      </c>
+      <c r="W5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Thread safe updation and parallel execution fixes
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06DCEA63-D5B2-447D-8B1E-66F1C7763AAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE38CAD-E65D-44E2-A941-567CF91809F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="217">
   <si>
     <t>titleValidationTest</t>
   </si>
@@ -56,12 +56,6 @@
   </si>
   <si>
     <t>System</t>
-  </si>
-  <si>
-    <t>Symx@4321</t>
-  </si>
-  <si>
-    <t>Symx@4322</t>
   </si>
   <si>
     <t>customerCategory</t>
@@ -746,7 +740,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -758,6 +752,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1128,226 +1123,226 @@
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="Y1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AC1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AV1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="AX1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="BE1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="BC1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="BE1" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="BF1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="BH1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BP1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="BT1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="BZ1" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:78" x14ac:dyDescent="0.25">
@@ -1357,8 +1352,8 @@
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
-        <v>10</v>
+      <c r="C2" s="7" t="s">
+        <v>76</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -1371,8 +1366,8 @@
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>11</v>
+      <c r="C3" s="7" t="s">
+        <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -1394,49 +1389,49 @@
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
       <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
         <v>32</v>
       </c>
-      <c r="F5" t="s">
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" t="s">
+        <v>188</v>
+      </c>
+      <c r="L5" t="s">
+        <v>189</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q5" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="S5" t="s">
         <v>34</v>
       </c>
-      <c r="I5" t="s">
+      <c r="T5" t="s">
         <v>38</v>
-      </c>
-      <c r="J5" t="s">
-        <v>190</v>
-      </c>
-      <c r="L5" t="s">
-        <v>191</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="S5" t="s">
-        <v>36</v>
-      </c>
-      <c r="T5" t="s">
-        <v>40</v>
       </c>
       <c r="U5">
         <v>91</v>
@@ -1445,43 +1440,43 @@
         <v>8521036250</v>
       </c>
       <c r="X5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AC5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="AD5">
         <v>123456</v>
       </c>
       <c r="AE5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AG5" t="s">
         <v>50</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AI5" t="s">
         <v>51</v>
       </c>
-      <c r="AG5" t="s">
+      <c r="AJ5" t="s">
         <v>52</v>
       </c>
-      <c r="AI5" t="s">
-        <v>53</v>
-      </c>
-      <c r="AJ5" t="s">
+      <c r="AK5" t="s">
         <v>54</v>
       </c>
-      <c r="AK5" t="s">
-        <v>56</v>
-      </c>
       <c r="AL5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="AM5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AN5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AO5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="AP5">
         <v>86501326</v>
@@ -1499,22 +1494,22 @@
         <v>123</v>
       </c>
       <c r="AU5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="AV5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="AX5" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>86</v>
+      </c>
+      <c r="AZ5" t="s">
         <v>87</v>
       </c>
-      <c r="AY5" t="s">
+      <c r="BA5" t="s">
         <v>88</v>
-      </c>
-      <c r="AZ5" t="s">
-        <v>89</v>
-      </c>
-      <c r="BA5" t="s">
-        <v>90</v>
       </c>
       <c r="BB5">
         <v>6260262069</v>
@@ -1523,75 +1518,75 @@
         <v>950959651959591</v>
       </c>
       <c r="BD5" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="BE5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="BF5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="BP5" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="BQ5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="BR5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="BS5">
         <v>75120365</v>
       </c>
       <c r="BT5" t="s">
+        <v>113</v>
+      </c>
+      <c r="BU5" t="s">
+        <v>114</v>
+      </c>
+      <c r="BV5" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="BU5" t="s">
+      <c r="BW5" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="BV5" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="BW5" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="BX5">
         <v>4102213652</v>
       </c>
       <c r="BY5" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="BZ5" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:78" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
       </c>
       <c r="F6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="G6" t="s">
+      <c r="L6" t="s">
         <v>175</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="Q6" t="s">
         <v>176</v>
-      </c>
-      <c r="L6" t="s">
-        <v>177</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>178</v>
       </c>
       <c r="U6">
         <v>1</v>
@@ -1600,43 +1595,43 @@
         <v>853210263</v>
       </c>
       <c r="X6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="Y6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="Z6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AB6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="AC6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="AD6">
         <v>5145656</v>
       </c>
       <c r="AE6" t="s">
+        <v>179</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>180</v>
+      </c>
+      <c r="AG6" t="s">
         <v>181</v>
       </c>
-      <c r="AF6" t="s">
-        <v>182</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>183</v>
-      </c>
       <c r="AI6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AN6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AO6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="AQ6">
         <v>63251</v>
@@ -1651,70 +1646,70 @@
         <v>36</v>
       </c>
       <c r="AV6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="AW6">
         <v>95959652</v>
       </c>
       <c r="AX6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AY6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="AZ6" t="s">
+        <v>87</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>187</v>
+      </c>
+      <c r="BE6" t="s">
         <v>89</v>
       </c>
-      <c r="BA6" t="s">
-        <v>90</v>
-      </c>
-      <c r="BD6" t="s">
-        <v>189</v>
-      </c>
-      <c r="BE6" t="s">
-        <v>91</v>
-      </c>
       <c r="BF6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="BG6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="BH6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="BI6" s="5">
         <v>596596596529656</v>
       </c>
       <c r="BK6" t="s">
+        <v>183</v>
+      </c>
+      <c r="BL6" t="s">
+        <v>184</v>
+      </c>
+      <c r="BM6" t="s">
         <v>185</v>
       </c>
-      <c r="BL6" t="s">
-        <v>186</v>
-      </c>
-      <c r="BM6" t="s">
-        <v>187</v>
-      </c>
       <c r="BR6" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="BS6">
         <v>959165656</v>
       </c>
       <c r="BT6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="BU6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="BV6" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="BW6" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="BZ6" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="BZ6" s="3" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.25">
@@ -1758,73 +1753,73 @@
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="M1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="P1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="R1" s="1" t="s">
+      <c r="V1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
@@ -1850,28 +1845,28 @@
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K2">
         <v>243</v>
@@ -1880,64 +1875,64 @@
         <v>8410236950</v>
       </c>
       <c r="M2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="N2" s="5">
         <v>62652965</v>
       </c>
       <c r="O2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="S2" s="5">
         <v>32616052</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="V2" s="3"/>
       <c r="W2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G3" t="s">
+        <v>141</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>145</v>
-      </c>
       <c r="I3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K3">
         <v>39</v>
@@ -1946,61 +1941,61 @@
         <v>9410236950</v>
       </c>
       <c r="M3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="N3" s="5">
         <v>8748019519</v>
       </c>
       <c r="O3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="R3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="S3" s="5">
         <v>740000562</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V3" s="3"/>
       <c r="W3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I4" t="s">
         <v>147</v>
-      </c>
-      <c r="I4" t="s">
-        <v>149</v>
       </c>
       <c r="K4">
         <v>40</v>
@@ -2009,63 +2004,63 @@
         <v>1024710236</v>
       </c>
       <c r="M4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="N4" s="5">
         <v>9595016</v>
       </c>
       <c r="O4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="R4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="S4" s="5">
         <v>521032154</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="V4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="W4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K5">
         <v>7</v>
@@ -2074,37 +2069,37 @@
         <v>6012354012</v>
       </c>
       <c r="M5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="N5" s="5">
         <v>654515332</v>
       </c>
       <c r="O5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="R5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="S5" s="5">
         <v>5490196</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="V5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="W5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Assert message methods implement with spinner wait mechanism
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE38CAD-E65D-44E2-A941-567CF91809F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA43E1D-F482-47CA-B8F6-395B959753F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="221">
   <si>
     <t>titleValidationTest</t>
   </si>
@@ -550,9 +550,6 @@
     <t>Resident</t>
   </si>
   <si>
-    <t>AlignMinds </t>
-  </si>
-  <si>
     <t>Technologies</t>
   </si>
   <si>
@@ -592,21 +589,6 @@
     <t>Branch</t>
   </si>
   <si>
-    <t>Shinitha</t>
-  </si>
-  <si>
-    <t>Thomas</t>
-  </si>
-  <si>
-    <t>10/05/1989</t>
-  </si>
-  <si>
-    <t>shinithat@cinque.ae</t>
-  </si>
-  <si>
-    <t>adminalignminds@gmail.com</t>
-  </si>
-  <si>
     <t>Food</t>
   </si>
   <si>
@@ -677,6 +659,36 @@
   </si>
   <si>
     <t>05/08/2015</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>Customer Saved Successfully</t>
+  </si>
+  <si>
+    <t>toastType</t>
+  </si>
+  <si>
+    <t>expectedMessages</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>ajayklmala@yahoo.in</t>
+  </si>
+  <si>
+    <t>10/05/1988</t>
+  </si>
+  <si>
+    <t>maruthamala</t>
+  </si>
+  <si>
+    <t>MindTree</t>
+  </si>
+  <si>
+    <t>adminmindstree@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -686,7 +698,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -714,11 +726,6 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF2A2A2A"/>
-      <name val="Poppins"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -740,7 +747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -749,9 +756,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1033,7 +1037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BZ7"/>
+  <dimension ref="A1:CB7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
@@ -1045,7 +1049,7 @@
     <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -1099,7 +1103,7 @@
     <col min="68" max="68" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="10" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="12" bestFit="1" customWidth="1"/>
     <col min="72" max="72" width="20" bestFit="1" customWidth="1"/>
     <col min="73" max="73" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="74" max="74" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -1107,9 +1111,11 @@
     <col min="76" max="76" width="12" bestFit="1" customWidth="1"/>
     <col min="77" max="77" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="78" max="78" width="60.140625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:80" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1344,36 +1350,42 @@
       <c r="BZ1" s="1" t="s">
         <v>111</v>
       </c>
+      <c r="CA1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="CB1" s="1" t="s">
+        <v>214</v>
+      </c>
     </row>
-    <row r="2" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:80" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" t="s">
         <v>76</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:80" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" t="s">
         <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:80" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1387,7 +1399,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:80" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>119</v>
       </c>
@@ -1416,13 +1428,13 @@
         <v>36</v>
       </c>
       <c r="J5" t="s">
-        <v>188</v>
+        <v>218</v>
       </c>
       <c r="L5" t="s">
-        <v>189</v>
+        <v>215</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>190</v>
+        <v>217</v>
       </c>
       <c r="Q5" s="4" t="s">
         <v>37</v>
@@ -1437,10 +1449,10 @@
         <v>91</v>
       </c>
       <c r="V5">
-        <v>8521036250</v>
+        <v>5632650050</v>
       </c>
       <c r="X5" t="s">
-        <v>191</v>
+        <v>216</v>
       </c>
       <c r="AC5" t="s">
         <v>47</v>
@@ -1536,7 +1548,7 @@
         <v>112</v>
       </c>
       <c r="BS5">
-        <v>75120365</v>
+        <v>9652695065</v>
       </c>
       <c r="BT5" t="s">
         <v>113</v>
@@ -1551,7 +1563,7 @@
         <v>116</v>
       </c>
       <c r="BX5">
-        <v>4102213652</v>
+        <v>6626026105</v>
       </c>
       <c r="BY5" s="3" t="s">
         <v>117</v>
@@ -1559,8 +1571,14 @@
       <c r="BZ5" s="3" t="s">
         <v>118</v>
       </c>
+      <c r="CA5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="CB5" t="s">
+        <v>212</v>
+      </c>
     </row>
-    <row r="6" spans="1:78" ht="19.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:80" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>128</v>
       </c>
@@ -1579,59 +1597,59 @@
       <c r="G6" t="s">
         <v>173</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" t="s">
+        <v>219</v>
+      </c>
+      <c r="L6" t="s">
         <v>174</v>
       </c>
-      <c r="L6" t="s">
+      <c r="Q6" t="s">
         <v>175</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>176</v>
       </c>
       <c r="U6">
         <v>1</v>
       </c>
       <c r="V6">
-        <v>853210263</v>
-      </c>
-      <c r="X6" t="s">
-        <v>192</v>
+        <v>113985403</v>
+      </c>
+      <c r="X6" s="6" t="s">
+        <v>220</v>
       </c>
       <c r="Y6" t="s">
         <v>171</v>
       </c>
       <c r="Z6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="AB6" t="s">
         <v>48</v>
       </c>
       <c r="AC6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AD6">
         <v>5145656</v>
       </c>
       <c r="AE6" t="s">
+        <v>178</v>
+      </c>
+      <c r="AF6" t="s">
         <v>179</v>
       </c>
-      <c r="AF6" t="s">
+      <c r="AG6" t="s">
         <v>180</v>
       </c>
-      <c r="AG6" t="s">
-        <v>181</v>
-      </c>
       <c r="AI6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AN6" t="s">
         <v>77</v>
       </c>
       <c r="AO6" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="AQ6">
         <v>63251</v>
@@ -1646,16 +1664,16 @@
         <v>36</v>
       </c>
       <c r="AV6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AW6">
         <v>95959652</v>
       </c>
       <c r="AX6" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="AY6" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="AZ6" t="s">
         <v>87</v>
@@ -1664,7 +1682,7 @@
         <v>88</v>
       </c>
       <c r="BD6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BE6" t="s">
         <v>89</v>
@@ -1673,31 +1691,31 @@
         <v>33</v>
       </c>
       <c r="BG6" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="BH6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BI6" s="5">
         <v>596596596529656</v>
       </c>
       <c r="BK6" t="s">
+        <v>182</v>
+      </c>
+      <c r="BL6" t="s">
         <v>183</v>
       </c>
-      <c r="BL6" t="s">
+      <c r="BM6" t="s">
         <v>184</v>
       </c>
-      <c r="BM6" t="s">
-        <v>185</v>
-      </c>
       <c r="BR6" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="BS6">
-        <v>959165656</v>
+        <v>5950656100</v>
       </c>
       <c r="BT6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="BU6" t="s">
         <v>48</v>
@@ -1711,8 +1729,14 @@
       <c r="BZ6" s="3" t="s">
         <v>118</v>
       </c>
+      <c r="CA6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="CB6" t="s">
+        <v>212</v>
+      </c>
     </row>
-    <row r="7" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:80" x14ac:dyDescent="0.25">
       <c r="I7" s="2"/>
     </row>
   </sheetData>
@@ -1762,37 +1786,37 @@
         <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>208</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>123</v>
@@ -1810,13 +1834,13 @@
         <v>109</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>126</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>127</v>
@@ -1866,7 +1890,7 @@
         <v>142</v>
       </c>
       <c r="I2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="K2">
         <v>243</v>
@@ -1881,7 +1905,7 @@
         <v>62652965</v>
       </c>
       <c r="O2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>149</v>
@@ -1914,7 +1938,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="D3" t="s">
         <v>134</v>
@@ -1947,7 +1971,7 @@
         <v>8748019519</v>
       </c>
       <c r="O3" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>150</v>
@@ -2010,7 +2034,7 @@
         <v>9595016</v>
       </c>
       <c r="O4" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>151</v>
@@ -2031,7 +2055,7 @@
         <v>167</v>
       </c>
       <c r="V4" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="W4" t="s">
         <v>118</v>
@@ -2075,7 +2099,7 @@
         <v>654515332</v>
       </c>
       <c r="O5" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>152</v>
@@ -2096,7 +2120,7 @@
         <v>168</v>
       </c>
       <c r="V5" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="W5" t="s">
         <v>118</v>

</xml_diff>

<commit_message>
Outward Remittance screen page object and test addition
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gopinath\IdeaProjects\SeleniumFrameworks\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA43E1D-F482-47CA-B8F6-395B959753F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CADBA10-30E3-4103-B15C-ADC83D9050AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6510" yWindow="570" windowWidth="11910" windowHeight="6525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -747,7 +747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -756,7 +756,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1612,7 +1611,7 @@
       <c r="V6">
         <v>113985403</v>
       </c>
-      <c r="X6" s="6" t="s">
+      <c r="X6" t="s">
         <v>220</v>
       </c>
       <c r="Y6" t="s">

</xml_diff>